<commit_message>
Update fact sheet: fix overstated claims and stale CAGR link
- Investor letter: replace "beats the basket in every scenario" (false in
  Bear, 0.27x) with the probability-weighted 1.34x KS-PME; state the
  Taiwan-shock holdco IRR vs Base explicitly; soften "uncorrelated" and
  "pays distributions first" to what the model supports
- Fact Sheet Data register now reads overlay-adjusted CAGRs (Weapons S,
  Consumer T); Saronic spotlight shows the modelled 27.3%, not raw 26%
- Saronic revenue growth stated as ~1,500% to ~$200M per source
- Key terms: add the munitions / FMS overlay row
- Model engine values unchanged; 21/21 checks pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011pVm4mKVqHD71s18HDPqrh
</commit_message>
<xml_diff>
--- a/models/Leviathan_PE_HOLDCO_Model_IC_VFinal_v3_Optimized_Letalis.xlsx
+++ b/models/Leviathan_PE_HOLDCO_Model_IC_VFinal_v3_Optimized_Letalis.xlsx
@@ -19620,7 +19620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N142"/>
+  <dimension ref="A1:N143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -20817,7 +20817,7 @@
       </c>
       <c r="G57" s="198" t="inlineStr">
         <is>
-          <t>Base CAGR</t>
+          <t>Base CAGR (as modelled, incl. overlays)</t>
         </is>
       </c>
       <c r="H57" s="198" t="inlineStr">
@@ -21368,8 +21368,8 @@
         <v>0.0075675675675675675</v>
       </c>
       <c r="G67" s="216">
-        <f>'Weapons Sleeve'!F12</f>
-        <v>0.26</v>
+        <f>'Weapons Sleeve'!S12</f>
+        <v>0.2725</v>
       </c>
       <c r="H67" s="242" t="inlineStr">
         <is>
@@ -21423,8 +21423,8 @@
         <v>0.03333333333333333</v>
       </c>
       <c r="G68" s="216">
-        <f>'Weapons Sleeve'!F13</f>
-        <v>0.24</v>
+        <f>'Weapons Sleeve'!S13</f>
+        <v>0.255</v>
       </c>
       <c r="H68" s="242" t="inlineStr">
         <is>
@@ -21478,8 +21478,8 @@
         <v>0.0025</v>
       </c>
       <c r="G69" s="216">
-        <f>'Weapons Sleeve'!F14</f>
-        <v>0.17</v>
+        <f>'Weapons Sleeve'!S14</f>
+        <v>0.195</v>
       </c>
       <c r="H69" s="242" t="inlineStr">
         <is>
@@ -21533,8 +21533,8 @@
         <v>0.01</v>
       </c>
       <c r="G70" s="216">
-        <f>'Weapons Sleeve'!F15</f>
-        <v>0.16</v>
+        <f>'Weapons Sleeve'!S15</f>
+        <v>0.175</v>
       </c>
       <c r="H70" s="242" t="inlineStr">
         <is>
@@ -21588,8 +21588,8 @@
         <v>0.019444444444444445</v>
       </c>
       <c r="G71" s="216">
-        <f>'Weapons Sleeve'!F16</f>
-        <v>0.12</v>
+        <f>'Weapons Sleeve'!S16</f>
+        <v>0.135</v>
       </c>
       <c r="H71" s="242" t="inlineStr">
         <is>
@@ -21643,8 +21643,8 @@
         <v>0.26666666666666666</v>
       </c>
       <c r="G72" s="216">
-        <f>'Weapons Sleeve'!F17</f>
-        <v>0.28</v>
+        <f>'Weapons Sleeve'!S17</f>
+        <v>0.30000000000000004</v>
       </c>
       <c r="H72" s="242" t="inlineStr">
         <is>
@@ -21698,8 +21698,8 @@
         <v>0.041666666666666664</v>
       </c>
       <c r="G73" s="216">
-        <f>'Weapons Sleeve'!F18</f>
-        <v>0.13</v>
+        <f>'Weapons Sleeve'!S18</f>
+        <v>0.1525</v>
       </c>
       <c r="H73" s="242" t="inlineStr">
         <is>
@@ -21753,8 +21753,8 @@
         <v>0.1</v>
       </c>
       <c r="G74" s="216">
-        <f>'Weapons Sleeve'!F19</f>
-        <v>0.13</v>
+        <f>'Weapons Sleeve'!S19</f>
+        <v>0.1525</v>
       </c>
       <c r="H74" s="242" t="inlineStr">
         <is>
@@ -21808,8 +21808,8 @@
         <v>0.03333333333333333</v>
       </c>
       <c r="G75" s="216">
-        <f>'Weapons Sleeve'!F20</f>
-        <v>0.14</v>
+        <f>'Weapons Sleeve'!S20</f>
+        <v>0.15250000000000002</v>
       </c>
       <c r="H75" s="242" t="inlineStr">
         <is>
@@ -21863,8 +21863,8 @@
         <v>0.0034653465346534654</v>
       </c>
       <c r="G76" s="216">
-        <f>'Consumer Sleeve'!F12</f>
-        <v>0.28</v>
+        <f>'Consumer Sleeve'!T12</f>
+        <v>0.29950000000000004</v>
       </c>
       <c r="H76" s="242" t="inlineStr">
         <is>
@@ -21918,8 +21918,8 @@
         <v>0.003118811881188119</v>
       </c>
       <c r="G77" s="216">
-        <f>'Consumer Sleeve'!F13</f>
-        <v>0.27</v>
+        <f>'Consumer Sleeve'!T13</f>
+        <v>0.28800000000000003</v>
       </c>
       <c r="H77" s="242" t="inlineStr">
         <is>
@@ -21973,8 +21973,8 @@
         <v>0.0065159574468085105</v>
       </c>
       <c r="G78" s="216">
-        <f>'Consumer Sleeve'!F14</f>
-        <v>0.22</v>
+        <f>'Consumer Sleeve'!T14</f>
+        <v>0.2385</v>
       </c>
       <c r="H78" s="242" t="inlineStr">
         <is>
@@ -22028,8 +22028,8 @@
         <v>0.0625</v>
       </c>
       <c r="G79" s="216">
-        <f>'Consumer Sleeve'!F15</f>
-        <v>0.14</v>
+        <f>'Consumer Sleeve'!T15</f>
+        <v>0.15700000000000003</v>
       </c>
       <c r="H79" s="242" t="inlineStr">
         <is>
@@ -22083,8 +22083,8 @@
         <v>0.014814814814814815</v>
       </c>
       <c r="G80" s="216">
-        <f>'Consumer Sleeve'!F16</f>
-        <v>0.07</v>
+        <f>'Consumer Sleeve'!T16</f>
+        <v>0.08750000000000001</v>
       </c>
       <c r="H80" s="242" t="inlineStr">
         <is>
@@ -22138,8 +22138,8 @@
         <v>0.06363636363636363</v>
       </c>
       <c r="G81" s="216">
-        <f>'Consumer Sleeve'!F17</f>
-        <v>0.2</v>
+        <f>'Consumer Sleeve'!T17</f>
+        <v>0.21550000000000002</v>
       </c>
       <c r="H81" s="242" t="inlineStr">
         <is>
@@ -22193,8 +22193,8 @@
         <v>0.0005833333333333334</v>
       </c>
       <c r="G82" s="216">
-        <f>'Consumer Sleeve'!F18</f>
-        <v>0.25</v>
+        <f>'Consumer Sleeve'!T18</f>
+        <v>0.266</v>
       </c>
       <c r="H82" s="242" t="inlineStr">
         <is>
@@ -22248,8 +22248,8 @@
         <v>0.004021447721179625</v>
       </c>
       <c r="G83" s="216">
-        <f>'Consumer Sleeve'!F19</f>
-        <v>0.15</v>
+        <f>'Consumer Sleeve'!T19</f>
+        <v>0.1625</v>
       </c>
       <c r="H83" s="242" t="inlineStr">
         <is>
@@ -22303,8 +22303,8 @@
         <v>0.0002830188679245283</v>
       </c>
       <c r="G84" s="216">
-        <f>'Consumer Sleeve'!F20</f>
-        <v>0.18</v>
+        <f>'Consumer Sleeve'!T20</f>
+        <v>0.199</v>
       </c>
       <c r="H84" s="242" t="inlineStr">
         <is>
@@ -23154,6 +23154,17 @@
       <c r="B142" s="258">
         <f>AVERAGE('Weapons Sleeve'!R12:R20)</f>
         <v>3.5555555555555554</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="200" t="inlineStr">
+        <is>
+          <t>Weapons munitions/FMS uplift per point Base / Bull / Bear / Shock</t>
+        </is>
+      </c>
+      <c r="B143" s="248" t="str">
+        <f>TEXT('Weapons Sleeve'!Q5,"0.0%")&amp;" / "&amp;TEXT('Weapons Sleeve'!Q6,"0.0%")&amp;" / "&amp;TEXT('Weapons Sleeve'!Q7,"0.0%")&amp;" / "&amp;TEXT('Weapons Sleeve'!Q8,"0.0%")</f>
+        <v>0.5% / 0.8% / 0.4% / 0.6%</v>
       </c>
     </row>
   </sheetData>
@@ -24461,7 +24472,7 @@
         </is>
       </c>
       <c r="B28" s="210">
-        <f>SUMPRODUCT(ISERROR('Holdco Summary'!B28:F86)*1)+SUMPRODUCT(ISERROR('Fund Economics'!B6:F49)*1)+SUMPRODUCT(ISERROR('Sleeve Economics'!B6:R53)*1)+SUMPRODUCT(ISERROR('Scenario Summary'!B6:F22)*1)+SUMPRODUCT(ISERROR('PME, DPI &amp; Sensitivity'!B13:F69)*1)+SUMPRODUCT(ISERROR('Fact Sheet Data'!B5:N143)*1)+SUMPRODUCT(ISERROR('IC Summary'!B6:F81)*1)</f>
+        <f>SUMPRODUCT(ISERROR('Holdco Summary'!B28:F86)*1)+SUMPRODUCT(ISERROR('Fund Economics'!B6:F49)*1)+SUMPRODUCT(ISERROR('Sleeve Economics'!B6:R53)*1)+SUMPRODUCT(ISERROR('Scenario Summary'!B6:F22)*1)+SUMPRODUCT(ISERROR('PME, DPI &amp; Sensitivity'!B13:F69)*1)+SUMPRODUCT(ISERROR('Fact Sheet Data'!B5:N144)*1)+SUMPRODUCT(ISERROR('IC Summary'!B6:F81)*1)</f>
         <v>0.0</v>
       </c>
       <c r="C28" s="207" t="str">

</xml_diff>